<commit_message>
Merged PR 2268: Merge MahadevProductB to master
Fixed issues in Progress Report
</commit_message>
<xml_diff>
--- a/src/main/resources/ProgressReport_Field_Values.xlsx
+++ b/src/main/resources/ProgressReport_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E4C57D-9E24-4DFB-8238-B6FC35D99452}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D495E921-21F6-4BA9-8D0F-861C9F2CE4C5}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" activeTab="1" xr2:uid="{2CF227FB-55E5-4154-93E7-6831A7625F64}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{2CF227FB-55E5-4154-93E7-6831A7625F64}"/>
   </bookViews>
   <sheets>
     <sheet name="Edition" sheetId="1" r:id="rId1"/>
@@ -135,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -143,6 +143,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,14 +462,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{756EB8E1-CDD7-4F47-B6A9-50B266C05D05}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="95.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="95.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -477,7 +480,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -488,7 +491,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -499,7 +502,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -510,7 +513,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -530,87 +533,87 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{165F264A-263B-4AE4-BE30-B37BD58F47A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="158" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="158" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4" t="s">
         <v>18</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="4">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="4">
         <v>-2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
       <c r="B7" t="s">
         <v>21</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="4" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed failed test cases and added new TC
</commit_message>
<xml_diff>
--- a/src/main/resources/ProgressReport_Field_Values.xlsx
+++ b/src/main/resources/ProgressReport_Field_Values.xlsx
@@ -1,24 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Product Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{612E53E8-2C44-4FD4-96B7-FEE0B9738D57}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC629CC9-44C2-40B9-A3B6-E0C94806CB53}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="2" xr2:uid="{2CF227FB-55E5-4154-93E7-6831A7625F64}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{2CF227FB-55E5-4154-93E7-6831A7625F64}"/>
   </bookViews>
   <sheets>
     <sheet name="Edition" sheetId="1" r:id="rId1"/>
-    <sheet name="ScheduleQuartelyCalendar" sheetId="3" r:id="rId2"/>
-    <sheet name="ScheduleAnnuallyCalendar" sheetId="4" r:id="rId3"/>
-    <sheet name="ScheduleSemiAnnually" sheetId="5" r:id="rId4"/>
-    <sheet name="ScheduleBiMonthly" sheetId="6" r:id="rId5"/>
-    <sheet name="Form Fields" sheetId="2" r:id="rId6"/>
+    <sheet name="PlanError" sheetId="10" r:id="rId2"/>
+    <sheet name="ObstacleError" sheetId="9" r:id="rId3"/>
+    <sheet name="KeyAccError" sheetId="8" r:id="rId4"/>
+    <sheet name="ErrorForAck" sheetId="7" r:id="rId5"/>
+    <sheet name="ScheduleQuartelyCalendar" sheetId="3" r:id="rId6"/>
+    <sheet name="ScheduleAnnuallyCalendar" sheetId="4" r:id="rId7"/>
+    <sheet name="ScheduleSemiAnnually" sheetId="5" r:id="rId8"/>
+    <sheet name="ScheduleBiMonthly" sheetId="6" r:id="rId9"/>
+    <sheet name="Form Fields" sheetId="2" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="44">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -612,408 +616,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9083A037-5F1C-4F1B-BC9C-BD3BCDD5C4F5}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B602DAF3-EA4C-4411-83F6-DC18D5FF0624}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE7AE48B-043F-4B46-920A-8E923AEFDF07}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D6733A2-29DF-4936-8F0F-DBCC59247680}">
-  <dimension ref="A1:K22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="3"/>
-    </row>
-    <row r="17" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I17" s="1"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="1"/>
-    </row>
-    <row r="18" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="7"/>
-    </row>
-    <row r="19" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-    </row>
-    <row r="20" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-    </row>
-    <row r="21" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="6"/>
-    </row>
-    <row r="22" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="6"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{165F264A-263B-4AE4-BE30-B37BD58F47A5}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1103,4 +706,643 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59CB41D5-3EB7-4F7C-BAA0-9B20DD4811C4}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="95.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D72F519A-34E9-47C6-868B-C146DEA726AE}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="95.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{439DE0DC-8395-49F9-9A33-3B799989CDF9}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="95.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EC6C784-F6B5-426A-A91D-7FBF6EF20C65}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="106" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9083A037-5F1C-4F1B-BC9C-BD3BCDD5C4F5}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B602DAF3-EA4C-4411-83F6-DC18D5FF0624}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE7AE48B-043F-4B46-920A-8E923AEFDF07}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D6733A2-29DF-4936-8F0F-DBCC59247680}">
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="3"/>
+    </row>
+    <row r="17" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I17" s="1"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="1"/>
+    </row>
+    <row r="18" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="7"/>
+    </row>
+    <row r="19" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+    </row>
+    <row r="20" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+    </row>
+    <row r="21" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="6"/>
+    </row>
+    <row r="22" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added new test cases for progress reprot
</commit_message>
<xml_diff>
--- a/src/main/resources/ProgressReport_Field_Values.xlsx
+++ b/src/main/resources/ProgressReport_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Product Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F82BA85F-D6BE-4B0E-ADAA-7000C92263A0}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCE5D659-0BDE-45A6-BFFA-0B30589978AD}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="6" xr2:uid="{2CF227FB-55E5-4154-93E7-6831A7625F64}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" firstSheet="7" activeTab="11" xr2:uid="{2CF227FB-55E5-4154-93E7-6831A7625F64}"/>
   </bookViews>
   <sheets>
     <sheet name="Edition" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="ScheduleSemiAnnually" sheetId="5" r:id="rId9"/>
     <sheet name="ScheduleBiMonthly" sheetId="6" r:id="rId10"/>
     <sheet name="Form Fields" sheetId="2" r:id="rId11"/>
+    <sheet name="ErrorForm" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="47">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -559,14 +560,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{756EB8E1-CDD7-4F47-B6A9-50B266C05D05}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="95.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="95.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -577,7 +578,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -588,7 +589,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -599,7 +600,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -610,7 +611,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -630,13 +631,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D6733A2-29DF-4936-8F0F-DBCC59247680}">
   <dimension ref="A1:K22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -647,7 +648,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -658,7 +659,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -669,7 +670,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -680,7 +681,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -691,7 +692,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -702,7 +703,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -713,37 +714,37 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.4">
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="9:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="9:11" x14ac:dyDescent="0.4">
       <c r="I17" s="1"/>
       <c r="J17" s="2"/>
       <c r="K17" s="1"/>
     </row>
-    <row r="18" spans="9:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="9:11" x14ac:dyDescent="0.4">
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="7"/>
     </row>
-    <row r="19" spans="9:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="9:11" x14ac:dyDescent="0.4">
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="9:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="9:11" x14ac:dyDescent="0.4">
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="9:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="9:11" x14ac:dyDescent="0.4">
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="9:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="9:11" x14ac:dyDescent="0.4">
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="6"/>
@@ -757,14 +758,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{165F264A-263B-4AE4-BE30-B37BD58F47A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.3828125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="158" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -775,7 +776,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -786,7 +787,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -797,7 +798,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -808,7 +809,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -819,7 +820,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -830,7 +831,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -838,6 +839,71 @@
         <v>21</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDF5434-4D12-4F2F-B98B-154625A9FF1F}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="4">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>22</v>
       </c>
     </row>
@@ -849,15 +915,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59CB41D5-3EB7-4F7C-BAA0-9B20DD4811C4}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="95.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="11.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.3046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="95.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.15234375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -868,7 +934,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -879,7 +945,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -890,7 +956,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -909,15 +975,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D72F519A-34E9-47C6-868B-C146DEA726AE}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="95.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="11.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.3046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="95.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.15234375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -928,7 +994,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -939,7 +1005,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -950,7 +1016,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -969,15 +1035,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{439DE0DC-8395-49F9-9A33-3B799989CDF9}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="95.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="11.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.3046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="95.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.15234375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -988,7 +1054,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -999,7 +1065,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1010,7 +1076,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -1029,13 +1095,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EC6C784-F6B5-426A-A91D-7FBF6EF20C65}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.3046875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="106" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1046,7 +1112,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1057,7 +1123,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1068,7 +1134,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -1087,13 +1153,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9083A037-5F1C-4F1B-BC9C-BD3BCDD5C4F5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1104,7 +1170,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -1115,7 +1181,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -1126,7 +1192,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -1137,7 +1203,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1148,7 +1214,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="15" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -1159,7 +1225,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="15" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1179,13 +1245,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8827C01F-82DB-4710-97BD-1D832235DF80}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1196,7 +1262,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -1207,7 +1273,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -1218,7 +1284,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -1229,7 +1295,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1240,7 +1306,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="15" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -1251,7 +1317,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="15" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1270,13 +1336,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B602DAF3-EA4C-4411-83F6-DC18D5FF0624}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1287,7 +1353,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -1298,7 +1364,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -1309,7 +1375,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -1320,7 +1386,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1331,7 +1397,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -1342,7 +1408,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1361,13 +1427,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE7AE48B-043F-4B46-920A-8E923AEFDF07}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1378,7 +1444,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -1389,7 +1455,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -1400,7 +1466,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -1411,7 +1477,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1422,7 +1488,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -1433,7 +1499,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>

</xml_diff>